<commit_message>
Store assets in subfolders
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC00CAD-7611-4AA1-8E08-772A3A7DCA30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324A20A8-1F1D-497D-BA11-3D9E1746D0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4189" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4204" uniqueCount="92">
   <si>
     <t>X</t>
   </si>
@@ -147,9 +147,6 @@
     <t>Sprite</t>
   </si>
   <si>
-    <t>Id</t>
-  </si>
-  <si>
     <t>Bit</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
   </si>
   <si>
     <t>Set when this cell contains a renderable wall</t>
-  </si>
-  <si>
-    <t>Id of block/sprite etc so up to 8 types of wall/sprite etc.</t>
   </si>
   <si>
     <t>Emu</t>
@@ -323,6 +317,12 @@
   <si>
     <t>Walk L 2</t>
   </si>
+  <si>
+    <t>Enemy</t>
+  </si>
+  <si>
+    <t>Block contains an enemy.</t>
+  </si>
 </sst>
 </file>
 
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -382,9 +382,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A21D89A8-E5EC-4EAA-92CE-B056DD4B8657}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -796,7 +793,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
         <v>8</v>
@@ -804,89 +801,121 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>40</v>
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>0</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -901,7 +930,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -909,7 +938,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -917,7 +946,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -925,7 +954,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -933,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -955,10 +984,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -966,13 +995,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -980,16 +1009,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -997,16 +1026,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1014,13 +1043,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1028,7 +1057,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1036,7 +1065,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1044,7 +1073,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1052,7 +1081,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1062,14 +1091,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F90467-4CD9-40FD-80C5-3B27CEDF7551}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
@@ -1088,8 +1117,11 @@
       <c r="F1" t="s">
         <v>32</v>
       </c>
+      <c r="G1" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>0</v>
       </c>
@@ -1108,8 +1140,11 @@
       <c r="F2" t="s">
         <v>26</v>
       </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1128,8 +1163,11 @@
       <c r="F3" t="s">
         <v>26</v>
       </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -1148,8 +1186,11 @@
       <c r="F4" t="s">
         <v>26</v>
       </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>1</v>
       </c>
@@ -1168,8 +1209,11 @@
       <c r="F5" t="s">
         <v>26</v>
       </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1188,8 +1232,11 @@
       <c r="F6" t="s">
         <v>26</v>
       </c>
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1208,8 +1255,11 @@
       <c r="F7" t="s">
         <v>26</v>
       </c>
+      <c r="G7" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1228,8 +1278,11 @@
       <c r="F8" t="s">
         <v>27</v>
       </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
@@ -1248,8 +1301,11 @@
       <c r="F9" t="s">
         <v>26</v>
       </c>
+      <c r="G9" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1268,8 +1324,11 @@
       <c r="F10" t="s">
         <v>26</v>
       </c>
+      <c r="G10" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -1288,13 +1347,16 @@
       <c r="F11" t="s">
         <v>26</v>
       </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
         <v>26</v>
@@ -1308,13 +1370,16 @@
       <c r="F13" t="s">
         <v>27</v>
       </c>
+      <c r="G13" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
@@ -1328,13 +1393,16 @@
       <c r="F14" t="s">
         <v>27</v>
       </c>
+      <c r="G14" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C15" t="s">
         <v>26</v>
@@ -1348,13 +1416,16 @@
       <c r="F15" t="s">
         <v>27</v>
       </c>
+      <c r="G15" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
         <v>26</v>
@@ -1366,6 +1437,9 @@
         <v>27</v>
       </c>
       <c r="F16" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14819,7 +14893,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4">
         <f>2*1024</f>
@@ -14828,7 +14902,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B5">
         <f>8*1024</f>
@@ -14837,7 +14911,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B6">
         <f>HEX2DEC("2000")</f>
@@ -14846,7 +14920,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B7">
         <v>4096</v>
@@ -14854,7 +14928,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B8">
         <v>1024</v>
@@ -14897,30 +14971,30 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" t="s">
         <v>45</v>
-      </c>
-      <c r="F1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" t="s">
-        <v>45</v>
-      </c>
-      <c r="J1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>16</v>
@@ -14947,7 +15021,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>640</v>
@@ -14977,7 +15051,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -15018,18 +15092,18 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>130</v>
@@ -15045,7 +15119,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B3">
         <v>140</v>
@@ -15065,7 +15139,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B4">
         <v>360</v>
@@ -15085,7 +15159,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B5">
         <v>360</v>
@@ -15105,7 +15179,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B6">
         <v>630</v>
@@ -15125,7 +15199,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B7">
         <v>410</v>
@@ -15145,7 +15219,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8">
         <v>530</v>
@@ -15165,7 +15239,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9">
         <v>570</v>

</xml_diff>

<commit_message>
Experiment with direct video mem access.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7440E436-38F8-4C02-8A4D-065CDC3A7715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABBAF53-852A-4090-A617-543C6D400C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="1725" yWindow="2880" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="9" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="9" r:id="rId2"/>
     <sheet name="AI States" sheetId="8" r:id="rId3"/>
     <sheet name="Tiles Type" sheetId="2" r:id="rId4"/>
-    <sheet name="Level 1" sheetId="1" r:id="rId5"/>
-    <sheet name="Memory Budget" sheetId="3" r:id="rId6"/>
-    <sheet name="Performance" sheetId="6" r:id="rId7"/>
-    <sheet name="Optimisation" sheetId="7" r:id="rId8"/>
+    <sheet name="Weapons" sheetId="10" r:id="rId5"/>
+    <sheet name="Level 1" sheetId="1" r:id="rId6"/>
+    <sheet name="Memory Budget" sheetId="3" r:id="rId7"/>
+    <sheet name="Performance" sheetId="6" r:id="rId8"/>
+    <sheet name="Optimisation" sheetId="7" r:id="rId9"/>
+    <sheet name="TIming" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4238" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4254" uniqueCount="122">
   <si>
     <t>X</t>
   </si>
@@ -379,6 +381,39 @@
   </si>
   <si>
     <t>Move away from player or sidestep.</t>
+  </si>
+  <si>
+    <t>Pistol</t>
+  </si>
+  <si>
+    <t>SMG</t>
+  </si>
+  <si>
+    <t>AK47</t>
+  </si>
+  <si>
+    <t>LMG</t>
+  </si>
+  <si>
+    <t>Soldger</t>
+  </si>
+  <si>
+    <t>Player start</t>
+  </si>
+  <si>
+    <t>No 32bit div</t>
+  </si>
+  <si>
+    <t>Bare loop</t>
+  </si>
+  <si>
+    <t>FPS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>EMU</t>
   </si>
 </sst>
 </file>
@@ -1213,6 +1248,52 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F426B8BD-42FE-4B91-BDF5-11A7679F9A78}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="8"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5235E873-4701-4130-881C-1F333236149A}">
   <dimension ref="A1:B5"/>
@@ -1757,6 +1838,51 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DFE4376-F190-41D3-ACAB-06DF87696190}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{750D9AD9-7C84-4603-A2EE-1597D412FCF4}">
   <dimension ref="A1:BM64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14477,7 +14603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5E0410-6B34-4610-813C-474405B474F7}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14594,7 +14720,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692BE518-AAC1-41EE-AD19-DC91CDF8547C}">
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14639,9 +14765,12 @@
       <c r="F2">
         <v>630</v>
       </c>
+      <c r="G2">
+        <v>10</v>
+      </c>
       <c r="H2">
-        <f>1000/F2</f>
-        <v>1.5873015873015872</v>
+        <f>1000/G2</f>
+        <v>100</v>
       </c>
       <c r="J2">
         <f>F2/B2</f>
@@ -14669,9 +14798,12 @@
       <c r="F3">
         <v>790</v>
       </c>
+      <c r="G3">
+        <v>30</v>
+      </c>
       <c r="H3">
-        <f>1000/F3</f>
-        <v>1.2658227848101267</v>
+        <f>1000/G3</f>
+        <v>33.333333333333336</v>
       </c>
       <c r="J3">
         <f>F3/B3</f>
@@ -14714,9 +14846,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB40D263-C04C-4263-859C-02DFCB83777C}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -14758,15 +14890,15 @@
         <v>140</v>
       </c>
       <c r="C3" s="4">
-        <f t="shared" ref="C3:C11" si="0">(B3/$B$2)-1</f>
+        <f t="shared" ref="C3:C12" si="0">(B3/$B$2)-1</f>
         <v>7.6923076923076872E-2</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E11" si="1">B3/40</f>
+        <f t="shared" ref="E3:E12" si="1">B3/40</f>
         <v>3.5</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F11" si="2">E3/3</f>
+        <f t="shared" ref="F3:F12" si="2">E3/3</f>
         <v>1.1666666666666667</v>
       </c>
     </row>
@@ -14928,6 +15060,26 @@
       <c r="F11">
         <f t="shared" si="2"/>
         <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12">
+        <v>610</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="shared" si="0"/>
+        <v>3.6923076923076925</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>15.25</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="2"/>
+        <v>5.083333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clear up unneeded sprites.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037DF8B9-4D02-4B3C-8E4C-512A77B1E457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B937672-58F4-42C1-B078-036389BCACB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="9" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4265" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4268" uniqueCount="135">
   <si>
     <t>X</t>
   </si>
@@ -445,6 +445,15 @@
   <si>
     <t>Vid mem</t>
   </si>
+  <si>
+    <t>Packed Bitmap</t>
+  </si>
+  <si>
+    <t>Full Spriite</t>
+  </si>
+  <si>
+    <t>Clipped Sprite</t>
+  </si>
 </sst>
 </file>
 
@@ -515,10 +524,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1141,7 +1150,7 @@
       <c r="A8">
         <v>9</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
       <c r="G8">
@@ -1161,7 +1170,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="9"/>
       <c r="G9">
         <v>8</v>
       </c>
@@ -1173,7 +1182,7 @@
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="9"/>
       <c r="C10" s="6"/>
       <c r="G10">
         <v>9</v>
@@ -1186,7 +1195,7 @@
       <c r="A11">
         <v>6</v>
       </c>
-      <c r="B11" s="8"/>
+      <c r="B11" s="9"/>
       <c r="C11" s="6"/>
       <c r="G11">
         <v>10</v>
@@ -1199,7 +1208,7 @@
       <c r="A12">
         <v>5</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="6"/>
@@ -1214,7 +1223,7 @@
       <c r="A13">
         <v>4</v>
       </c>
-      <c r="B13" s="8"/>
+      <c r="B13" s="9"/>
       <c r="C13" s="6"/>
       <c r="G13">
         <v>12</v>
@@ -1227,7 +1236,7 @@
       <c r="A14">
         <v>3</v>
       </c>
-      <c r="B14" s="8"/>
+      <c r="B14" s="9"/>
       <c r="C14" s="6"/>
       <c r="G14">
         <v>13</v>
@@ -1240,7 +1249,7 @@
       <c r="A15">
         <v>2</v>
       </c>
-      <c r="B15" s="8"/>
+      <c r="B15" s="9"/>
       <c r="C15" s="6"/>
       <c r="G15">
         <v>14</v>
@@ -1253,7 +1262,7 @@
       <c r="A16">
         <v>1</v>
       </c>
-      <c r="B16" s="8"/>
+      <c r="B16" s="9"/>
       <c r="C16" s="6"/>
       <c r="G16">
         <v>15</v>
@@ -1266,7 +1275,7 @@
       <c r="A17">
         <v>0</v>
       </c>
-      <c r="B17" s="8"/>
+      <c r="B17" s="9"/>
       <c r="C17" s="6"/>
     </row>
   </sheetData>
@@ -1281,35 +1290,35 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F426B8BD-42FE-4B91-BDF5-11A7679F9A78}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="9"/>
-    <col min="5" max="5" width="9.140625" style="9"/>
+    <col min="3" max="3" width="9.140625" style="8"/>
+    <col min="5" max="5" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="8"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>120</v>
       </c>
       <c r="D2" t="s">
         <v>119</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1320,15 +1329,15 @@
       <c r="B3">
         <v>32000</v>
       </c>
-      <c r="C3" s="9">
-        <f>1000/B3</f>
+      <c r="C3" s="8">
+        <f t="shared" ref="C3:C12" si="0">1000/B3</f>
         <v>3.125E-2</v>
       </c>
       <c r="D3">
         <v>13000</v>
       </c>
-      <c r="E3" s="9">
-        <f>1000/D3</f>
+      <c r="E3" s="8">
+        <f t="shared" ref="E3:E17" si="1">1000/D3</f>
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
@@ -1339,16 +1348,20 @@
       <c r="B4">
         <v>17610</v>
       </c>
-      <c r="C4" s="9">
-        <f>1000/B4</f>
+      <c r="C4" s="8">
+        <f t="shared" si="0"/>
         <v>5.6785917092561047E-2</v>
       </c>
       <c r="D4">
         <v>310</v>
       </c>
-      <c r="E4" s="9">
-        <f>1000/D4</f>
+      <c r="E4" s="8">
+        <f t="shared" si="1"/>
         <v>3.225806451612903</v>
+      </c>
+      <c r="F4" s="8">
+        <f>E4-E3</f>
+        <v>3.1488833746898259</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1358,16 +1371,20 @@
       <c r="B5">
         <v>850</v>
       </c>
-      <c r="C5" s="9">
-        <f>1000/B5</f>
+      <c r="C5" s="8">
+        <f t="shared" si="0"/>
         <v>1.1764705882352942</v>
       </c>
       <c r="D5">
         <v>32</v>
       </c>
-      <c r="E5" s="9">
-        <f>1000/D5</f>
+      <c r="E5" s="8">
+        <f t="shared" si="1"/>
         <v>31.25</v>
+      </c>
+      <c r="F5" s="8">
+        <f>E5-(E4+E3)</f>
+        <v>27.947270471464019</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1377,16 +1394,20 @@
       <c r="B6">
         <v>29000</v>
       </c>
-      <c r="C6" s="9">
-        <f>1000/B6</f>
+      <c r="C6" s="8">
+        <f t="shared" si="0"/>
         <v>3.4482758620689655E-2</v>
       </c>
       <c r="D6">
         <v>12700</v>
       </c>
-      <c r="E6" s="9">
-        <f>1000/D6</f>
+      <c r="E6" s="8">
+        <f t="shared" si="1"/>
         <v>7.874015748031496E-2</v>
+      </c>
+      <c r="F6" s="8">
+        <f>E6-E3</f>
+        <v>1.8170805572380322E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1396,16 +1417,20 @@
       <c r="B7">
         <v>32000</v>
       </c>
-      <c r="C7" s="9">
-        <f>1000/B7</f>
+      <c r="C7" s="8">
+        <f t="shared" si="0"/>
         <v>3.125E-2</v>
       </c>
       <c r="D7">
         <v>2406</v>
       </c>
-      <c r="E7" s="9">
-        <f>1000/D7</f>
+      <c r="E7" s="8">
+        <f t="shared" si="1"/>
         <v>0.41562759767248547</v>
+      </c>
+      <c r="F7" s="8">
+        <f>E7-E3</f>
+        <v>0.33870452074940854</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1415,16 +1440,20 @@
       <c r="B8">
         <v>32000</v>
       </c>
-      <c r="C8" s="9">
-        <f>1000/B8</f>
+      <c r="C8" s="8">
+        <f t="shared" si="0"/>
         <v>3.125E-2</v>
       </c>
       <c r="D8">
         <v>365</v>
       </c>
-      <c r="E8" s="9">
-        <f>1000/D8</f>
+      <c r="E8" s="8">
+        <f t="shared" si="1"/>
         <v>2.7397260273972601</v>
+      </c>
+      <c r="F8" s="8">
+        <f>E8-E3</f>
+        <v>2.662802950474183</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1434,17 +1463,22 @@
       <c r="B9">
         <v>2600</v>
       </c>
-      <c r="C9" s="9">
-        <f>1000/B9</f>
+      <c r="C9" s="8">
+        <f t="shared" si="0"/>
         <v>0.38461538461538464</v>
       </c>
       <c r="D9">
         <v>22</v>
       </c>
-      <c r="E9" s="9">
-        <f>1000/D9</f>
+      <c r="E9" s="8">
+        <f t="shared" si="1"/>
         <v>45.454545454545453</v>
       </c>
+      <c r="F9" s="8">
+        <f>E9-(E4+E3)</f>
+        <v>42.151815926009476</v>
+      </c>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1453,16 +1487,20 @@
       <c r="B10">
         <v>2800</v>
       </c>
-      <c r="C10" s="9">
-        <f>1000/B10</f>
+      <c r="C10" s="8">
+        <f t="shared" si="0"/>
         <v>0.35714285714285715</v>
       </c>
       <c r="D10">
         <v>24</v>
       </c>
-      <c r="E10" s="9">
-        <f>1000/D10</f>
+      <c r="E10" s="8">
+        <f t="shared" si="1"/>
         <v>41.666666666666664</v>
+      </c>
+      <c r="F10" s="8">
+        <f>E9-E10</f>
+        <v>3.787878787878789</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1472,16 +1510,20 @@
       <c r="B11">
         <v>3800</v>
       </c>
-      <c r="C11" s="9">
-        <f>1000/B11</f>
+      <c r="C11" s="8">
+        <f t="shared" si="0"/>
         <v>0.26315789473684209</v>
       </c>
       <c r="D11">
         <v>38</v>
       </c>
-      <c r="E11" s="9">
-        <f>1000/D11</f>
+      <c r="E11" s="8">
+        <f t="shared" si="1"/>
         <v>26.315789473684209</v>
+      </c>
+      <c r="F11" s="8">
+        <f>E9-E11</f>
+        <v>19.138755980861244</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1491,16 +1533,20 @@
       <c r="B12">
         <v>4562</v>
       </c>
-      <c r="C12" s="9">
-        <f>1000/B12</f>
+      <c r="C12" s="8">
+        <f t="shared" si="0"/>
         <v>0.21920210434020165</v>
       </c>
       <c r="D12">
         <v>47</v>
       </c>
-      <c r="E12" s="9">
-        <f>1000/D12</f>
+      <c r="E12" s="8">
+        <f t="shared" si="1"/>
         <v>21.276595744680851</v>
+      </c>
+      <c r="F12" s="8">
+        <f>E9-E12</f>
+        <v>24.177949709864603</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1510,11 +1556,11 @@
       <c r="D13">
         <v>12</v>
       </c>
-      <c r="E13" s="9">
-        <f>1000/D13</f>
+      <c r="E13" s="8">
+        <f t="shared" si="1"/>
         <v>83.333333333333329</v>
       </c>
-      <c r="G13" s="9"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1523,11 +1569,51 @@
       <c r="D14">
         <v>20</v>
       </c>
-      <c r="E14" s="9">
-        <f>1000/D14</f>
+      <c r="E14" s="8">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="F14" s="9"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D15">
+        <v>23</v>
+      </c>
+      <c r="E15" s="8">
+        <f t="shared" si="1"/>
+        <v>43.478260869565219</v>
+      </c>
+      <c r="F15" s="8">
+        <f>E15-E14</f>
+        <v>-6.5217391304347814</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16">
+        <v>14</v>
+      </c>
+      <c r="E16" s="8">
+        <f t="shared" si="1"/>
+        <v>71.428571428571431</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>134</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="E17" s="8">
+        <f t="shared" si="1"/>
+        <v>62.5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add PC build, AI fixes, weapon tuning.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4597E5-22BA-410B-B00C-7C7B7FF13FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5855B3-311B-49F3-9B79-9EC0927EA24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4357" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4443" uniqueCount="179">
   <si>
     <t>X</t>
   </si>
@@ -332,15 +332,6 @@
     <t>Wall types</t>
   </si>
   <si>
-    <t>Default wall</t>
-  </si>
-  <si>
-    <t>Dark Wall</t>
-  </si>
-  <si>
-    <t>Bars</t>
-  </si>
-  <si>
     <t>Enemy Types</t>
   </si>
   <si>
@@ -510,6 +501,90 @@
   </si>
   <si>
     <t>Pickups</t>
+  </si>
+  <si>
+    <t>SOLID (default)</t>
+  </si>
+  <si>
+    <t>DARK</t>
+  </si>
+  <si>
+    <t>WINDOW</t>
+  </si>
+  <si>
+    <t>ARCH</t>
+  </si>
+  <si>
+    <t>UNLOCKED_DOOR</t>
+  </si>
+  <si>
+    <t>BARS</t>
+  </si>
+  <si>
+    <t>VOID</t>
+  </si>
+  <si>
+    <t>LOCKED_DOOR</t>
+  </si>
+  <si>
+    <t>!</t>
+  </si>
+  <si>
+    <t>SIGN</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>LIGHT</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
+    <t>PIPES</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>SHELF</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>|</t>
+  </si>
+  <si>
+    <t>PILLAR</t>
+  </si>
+  <si>
+    <t>SWITCH</t>
+  </si>
+  <si>
+    <t>SHOOTABLE</t>
+  </si>
+  <si>
+    <t>Decorations</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Reserved</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Map</t>
+  </si>
+  <si>
+    <t>Item</t>
   </si>
 </sst>
 </file>
@@ -520,7 +595,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -544,6 +619,21 @@
       <sz val="11"/>
       <color rgb="FF569CD6"/>
       <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cascadia Code"/>
       <family val="3"/>
     </font>
   </fonts>
@@ -573,7 +663,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -590,15 +680,21 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill>
@@ -617,9 +713,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
+          <bgColor theme="8" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -681,103 +780,9 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFF00"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1121,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A21D89A8-E5EC-4EAA-92CE-B056DD4B8657}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -1132,13 +1137,20 @@
     <col min="6" max="6" width="9.85546875" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1151,32 +1163,47 @@
       <c r="G1">
         <v>0</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
       <c r="I1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K1" t="s">
         <v>94</v>
       </c>
-      <c r="K1" t="s">
-        <v>97</v>
-      </c>
-      <c r="L1">
-        <v>0</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="L1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1">
+        <v>0</v>
+      </c>
+      <c r="N1" t="s">
         <v>61</v>
       </c>
-      <c r="O1" t="s">
-        <v>153</v>
-      </c>
-      <c r="P1">
-        <v>0</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="P1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q1">
+        <v>0</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="S1" t="s">
+        <v>144</v>
+      </c>
+      <c r="V1" t="s">
+        <v>176</v>
+      </c>
+      <c r="W1" t="s">
+        <v>177</v>
+      </c>
+      <c r="X1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>15</v>
       </c>
@@ -1189,26 +1216,44 @@
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" t="s">
         <v>4</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
-      </c>
-      <c r="L2">
+        <v>152</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>79</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>1</v>
       </c>
-      <c r="Q2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="S2" t="s">
+        <v>145</v>
+      </c>
+      <c r="U2" t="s">
+        <v>172</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>14</v>
       </c>
@@ -1221,26 +1266,41 @@
       <c r="G3">
         <v>2</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" t="s">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L3">
+        <v>153</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3">
         <v>2</v>
       </c>
-      <c r="M3" t="s">
-        <v>98</v>
-      </c>
-      <c r="P3">
+      <c r="N3" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3">
         <v>2</v>
       </c>
-      <c r="Q3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R3" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="S3" t="s">
+        <v>146</v>
+      </c>
+      <c r="V3">
+        <v>1</v>
+      </c>
+      <c r="W3">
+        <v>2</v>
+      </c>
+      <c r="X3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>13</v>
       </c>
@@ -1253,26 +1313,41 @@
       <c r="G4">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" t="s">
         <v>2</v>
       </c>
       <c r="I4" t="s">
-        <v>11</v>
-      </c>
-      <c r="L4">
+        <v>154</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4">
         <v>3</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>81</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>3</v>
       </c>
-      <c r="Q4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R4" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="S4" t="s">
+        <v>148</v>
+      </c>
+      <c r="V4">
+        <v>2</v>
+      </c>
+      <c r="W4">
+        <v>3</v>
+      </c>
+      <c r="X4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>12</v>
       </c>
@@ -1285,20 +1360,32 @@
       <c r="G5">
         <v>4</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" t="s">
         <v>3</v>
       </c>
       <c r="I5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L5">
+        <v>155</v>
+      </c>
+      <c r="M5">
         <v>4</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="V5">
+        <v>3</v>
+      </c>
+      <c r="W5">
+        <v>4</v>
+      </c>
+      <c r="X5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>11</v>
       </c>
@@ -1311,20 +1398,32 @@
       <c r="G6">
         <v>5</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" t="s">
         <v>5</v>
       </c>
       <c r="I6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6">
+        <v>171</v>
+      </c>
+      <c r="M6">
         <v>5</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R6" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="V6">
+        <v>4</v>
+      </c>
+      <c r="W6">
+        <v>5</v>
+      </c>
+      <c r="X6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>10</v>
       </c>
@@ -1337,183 +1436,282 @@
       <c r="G7">
         <v>6</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" t="s">
         <v>19</v>
       </c>
       <c r="I7" t="s">
-        <v>96</v>
-      </c>
-      <c r="L7">
+        <v>156</v>
+      </c>
+      <c r="M7">
         <v>6</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="V7">
+        <v>5</v>
+      </c>
+      <c r="W7">
+        <v>6</v>
+      </c>
+      <c r="X7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>6</v>
       </c>
       <c r="G8">
         <v>7</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" t="s">
         <v>21</v>
       </c>
       <c r="I8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8">
+        <v>157</v>
+      </c>
+      <c r="M8">
         <v>7</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="R8" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="V8">
+        <v>6</v>
+      </c>
+      <c r="W8">
+        <v>7</v>
+      </c>
+      <c r="X8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="11"/>
       <c r="G9">
         <v>8</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>144</v>
+      <c r="H9" t="s">
+        <v>141</v>
       </c>
       <c r="I9" t="s">
-        <v>152</v>
-      </c>
-      <c r="L9">
+        <v>158</v>
+      </c>
+      <c r="M9">
         <v>8</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V9">
+        <v>7</v>
+      </c>
+      <c r="W9">
+        <v>8</v>
+      </c>
+      <c r="X9" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="11"/>
       <c r="C10" s="6"/>
       <c r="G10">
         <v>9</v>
       </c>
-      <c r="L10">
+      <c r="H10" t="s">
+        <v>159</v>
+      </c>
+      <c r="I10" t="s">
+        <v>160</v>
+      </c>
+      <c r="M10">
         <v>9</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>6</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="11"/>
       <c r="C11" s="6"/>
       <c r="G11">
         <v>10</v>
       </c>
-      <c r="L11">
+      <c r="H11" t="s">
+        <v>161</v>
+      </c>
+      <c r="I11" t="s">
+        <v>162</v>
+      </c>
+      <c r="M11">
         <v>10</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="6"/>
       <c r="G12">
         <v>11</v>
       </c>
-      <c r="L12">
+      <c r="H12" t="s">
+        <v>163</v>
+      </c>
+      <c r="I12" t="s">
+        <v>164</v>
+      </c>
+      <c r="M12">
         <v>11</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="11"/>
       <c r="C13" s="6"/>
       <c r="G13">
         <v>12</v>
       </c>
-      <c r="L13">
+      <c r="H13" t="s">
+        <v>165</v>
+      </c>
+      <c r="I13" t="s">
+        <v>166</v>
+      </c>
+      <c r="M13">
         <v>12</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3</v>
       </c>
-      <c r="B14" s="10"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="6"/>
       <c r="G14">
         <v>13</v>
       </c>
-      <c r="L14">
+      <c r="H14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" t="s">
+        <v>167</v>
+      </c>
+      <c r="M14">
         <v>13</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="11"/>
       <c r="C15" s="6"/>
       <c r="G15">
         <v>14</v>
       </c>
-      <c r="L15">
+      <c r="H15" t="s">
+        <v>168</v>
+      </c>
+      <c r="I15" t="s">
+        <v>169</v>
+      </c>
+      <c r="M15">
         <v>14</v>
       </c>
-      <c r="P15">
+      <c r="Q15">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="V15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="11"/>
       <c r="C16" s="6"/>
       <c r="G16">
         <v>15</v>
       </c>
-      <c r="L16">
+      <c r="H16" t="s">
+        <v>142</v>
+      </c>
+      <c r="I16" t="s">
+        <v>170</v>
+      </c>
+      <c r="M16">
         <v>15</v>
       </c>
-      <c r="P16">
+      <c r="Q16">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="V16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>0</v>
       </c>
-      <c r="B17" s="10"/>
+      <c r="B17" s="11"/>
       <c r="C17" s="6"/>
+      <c r="V17">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1538,32 +1736,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10" t="s">
+      <c r="B1" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="10"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B3">
         <v>32000</v>
@@ -1582,7 +1780,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B4">
         <v>850</v>
@@ -1609,7 +1807,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B5">
         <v>29000</v>
@@ -1636,7 +1834,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B6">
         <v>32000</v>
@@ -1663,7 +1861,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B7">
         <v>32000</v>
@@ -1694,7 +1892,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B8">
         <v>2600</v>
@@ -1721,7 +1919,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B9">
         <v>2800</v>
@@ -1744,7 +1942,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B10">
         <v>3800</v>
@@ -1798,7 +1996,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D12">
         <v>9</v>
@@ -1814,7 +2012,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D13">
         <v>15</v>
@@ -1838,7 +2036,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D14">
         <v>8</v>
@@ -1850,7 +2048,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D15">
         <v>11</v>
@@ -1965,10 +2163,10 @@
         <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2013,13 +2211,13 @@
         <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2044,13 +2242,13 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" t="s">
         <v>105</v>
-      </c>
-      <c r="E8" t="s">
-        <v>106</v>
-      </c>
-      <c r="F8" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2061,13 +2259,13 @@
         <v>71</v>
       </c>
       <c r="D9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" t="s">
         <v>107</v>
-      </c>
-      <c r="E9" t="s">
-        <v>109</v>
-      </c>
-      <c r="F9" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2081,7 +2279,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F90467-4CD9-40FD-80C5-3B27CEDF7551}">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -2137,7 +2335,7 @@
       <c r="G2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="10" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2163,7 +2361,7 @@
       <c r="G3" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="M3" s="10" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2189,7 +2387,7 @@
       <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="10" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2215,7 +2413,7 @@
       <c r="G5" t="s">
         <v>24</v>
       </c>
-      <c r="M5" s="11" t="s">
+      <c r="M5" s="10" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2241,7 +2439,7 @@
       <c r="G6" t="s">
         <v>24</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="M6" s="10" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2267,16 +2465,16 @@
       <c r="G7" t="s">
         <v>24</v>
       </c>
-      <c r="M7" s="11" t="s">
+      <c r="M7" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -2293,8 +2491,8 @@
       <c r="G8" t="s">
         <v>24</v>
       </c>
-      <c r="M8" s="11" t="s">
-        <v>135</v>
+      <c r="M8" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -2311,7 +2509,7 @@
         <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
         <v>24</v>
@@ -2319,12 +2517,12 @@
       <c r="G9" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="11" t="s">
-        <v>136</v>
+      <c r="M9" s="10" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="12" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
@@ -2345,12 +2543,12 @@
       <c r="G10" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="11" t="s">
-        <v>137</v>
+      <c r="M10" s="10" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B11" t="s">
@@ -2371,182 +2569,203 @@
       <c r="G11" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="11" t="s">
+      <c r="M11" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B12" t="s">
+        <v>160</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M12" s="11" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" t="s">
-        <v>25</v>
-      </c>
-      <c r="M13" s="11" t="s">
+    <row r="16" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" t="s">
-        <v>91</v>
-      </c>
-      <c r="C14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" t="s">
-        <v>25</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" t="s">
-        <v>25</v>
-      </c>
-      <c r="M15" s="11" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>167</v>
       </c>
       <c r="C16" t="s">
         <v>24</v>
       </c>
       <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
         <v>24</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" t="s">
+        <v>24</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="B17" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" t="s">
         <v>25</v>
       </c>
-      <c r="F16" t="s">
+      <c r="E17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" t="s">
+        <v>24</v>
+      </c>
+      <c r="M17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" t="s">
         <v>25</v>
       </c>
-      <c r="G16" t="s">
+      <c r="D18" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M17" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B18" t="s">
-        <v>147</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>24</v>
       </c>
-      <c r="D18" t="s">
+      <c r="F18" t="s">
         <v>24</v>
-      </c>
-      <c r="E18" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" t="s">
-        <v>25</v>
       </c>
       <c r="G18" t="s">
         <v>24</v>
       </c>
       <c r="M18" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B19" t="s">
-        <v>148</v>
-      </c>
-      <c r="C19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" t="s">
-        <v>24</v>
-      </c>
-      <c r="M19" s="11" t="s">
+      <c r="M19" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>137</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
-        <v>149</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
         <v>24</v>
@@ -2561,18 +2780,18 @@
         <v>25</v>
       </c>
       <c r="G20" t="s">
-        <v>24</v>
-      </c>
-      <c r="M20" s="11" t="s">
-        <v>144</v>
+        <v>25</v>
+      </c>
+      <c r="M20" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>138</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>151</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
         <v>24</v>
@@ -2587,18 +2806,18 @@
         <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>24</v>
-      </c>
-      <c r="M21" t="s">
-        <v>145</v>
+        <v>25</v>
+      </c>
+      <c r="M21" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>139</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>150</v>
+        <v>92</v>
       </c>
       <c r="C22" t="s">
         <v>24</v>
@@ -2613,18 +2832,18 @@
         <v>25</v>
       </c>
       <c r="G22" t="s">
-        <v>24</v>
-      </c>
-      <c r="M22" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
+      </c>
+      <c r="M22" s="10" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>140</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>150</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
         <v>24</v>
@@ -2639,44 +2858,23 @@
         <v>25</v>
       </c>
       <c r="G23" t="s">
-        <v>24</v>
-      </c>
-      <c r="M23" s="11" t="s">
-        <v>1</v>
+        <v>25</v>
+      </c>
+      <c r="M23" s="10" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" t="s">
-        <v>150</v>
-      </c>
-      <c r="C24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="M24" t="s">
         <v>25</v>
-      </c>
-      <c r="F24" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" t="s">
-        <v>24</v>
-      </c>
-      <c r="M24" s="11" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="B25" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
         <v>24</v>
@@ -2694,63 +2892,228 @@
         <v>24</v>
       </c>
       <c r="M25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M26" t="s">
+      <c r="F26" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" t="s">
+        <v>24</v>
+      </c>
+      <c r="M26" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M27" s="11">
-        <v>0</v>
+      <c r="C27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" t="s">
+        <v>24</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B28" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" t="s">
+        <v>24</v>
+      </c>
       <c r="M28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" t="s">
+        <v>147</v>
+      </c>
+      <c r="C29" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" t="s">
+        <v>24</v>
+      </c>
       <c r="M29">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" t="s">
+        <v>24</v>
+      </c>
       <c r="M30">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" t="s">
+        <v>24</v>
+      </c>
       <c r="M31">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" t="s">
+        <v>24</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" t="s">
+        <v>24</v>
+      </c>
       <c r="M32">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="13:13" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="M33">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="13:13" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A34"/>
       <c r="M34">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="13:13" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A35"/>
       <c r="M35">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="13:13" x14ac:dyDescent="0.25">
-      <c r="M36">
         <v>9</v>
       </c>
+    </row>
+    <row r="36" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A36"/>
+    </row>
+    <row r="37" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A37"/>
+    </row>
+    <row r="38" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A38"/>
+    </row>
+    <row r="39" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A39"/>
+    </row>
+    <row r="40" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A40"/>
+    </row>
+    <row r="41" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A41"/>
+    </row>
+    <row r="42" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A42"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2768,15 +3131,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s">
         <v>79</v>
@@ -2784,15 +3147,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
         <v>81</v>
@@ -4077,7 +4440,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA7" s="2">
         <v>0</v>
@@ -4089,7 +4452,7 @@
         <v>0</v>
       </c>
       <c r="AD7" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE7" s="2" t="s">
         <v>0</v>
@@ -4195,7 +4558,7 @@
       </c>
       <c r="BM7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XX00G00XXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX0XX10G02XXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="8" spans="1:65" x14ac:dyDescent="0.25">
@@ -5061,7 +5424,7 @@
         <v>0</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="Y12" s="2">
         <v>0</v>
@@ -5457,7 +5820,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="Y14" s="2" t="s">
         <v>0</v>
@@ -15486,40 +15849,40 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:BL64">
-    <cfRule type="containsText" dxfId="20" priority="12" operator="containsText" text="X">
+    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="X">
       <formula>NOT(ISERROR(SEARCH("X",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:BL1048576">
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+      <formula>"D"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"F"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>"E"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="9" operator="equal">
       <formula>"T"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
       <formula>"P"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="11" operator="equal">
       <formula>"W"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
-      <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15831,7 +16194,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B10">
         <v>600</v>
@@ -15851,7 +16214,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B11">
         <v>600</v>
@@ -15871,7 +16234,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B12">
         <v>610</v>
@@ -15891,7 +16254,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E13">
         <v>8</v>
@@ -15919,7 +16282,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E15">
         <v>12</v>

</xml_diff>